<commit_message>
Completed Booking and Status Updation
</commit_message>
<xml_diff>
--- a/backend/data.xlsx
+++ b/backend/data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\Practice\MERN\event-booking-and-ticketing\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C31DE33-DC69-432C-9D65-A495C58A225D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B58A73-5DBA-4A9A-8863-0B23D8B7D37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1170B748-74A8-4F51-B865-6844E1F4A4D7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1170B748-74A8-4F51-B865-6844E1F4A4D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Rating" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
   <si>
     <t>6aabaf9b1896552dfac49667</t>
   </si>
@@ -136,12 +137,71 @@
   <si>
     <t>2026-12-17T23:00:00.000Z</t>
   </si>
+  <si>
+    <t>Booking Lifecycle</t>
+  </si>
+  <si>
+    <t>Update Payment</t>
+  </si>
+  <si>
+    <t>Update Despatch</t>
+  </si>
+  <si>
+    <t>Difficulty Level</t>
+  </si>
+  <si>
+    <t>Advanced (8 / 10)</t>
+  </si>
+  <si>
+    <t>Performance Score</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>LC</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">You are firmly writing production-grade enterprise logic independently. The step up to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>excellent</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is simply sharpening code hygiene and catch-points before running execution.</t>
+    </r>
+  </si>
+  <si>
+    <t>Intermediate (6.5 / 10)</t>
+  </si>
+  <si>
+    <t>Update Receive Status</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,6 +243,19 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -219,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -233,6 +306,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,4 +770,87 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C25416-15F1-45E5-92CA-5DD08DB17583}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="147.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
cancellation and inventory rollback completed
</commit_message>
<xml_diff>
--- a/backend/data.xlsx
+++ b/backend/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\Practice\MERN\event-booking-and-ticketing\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B58A73-5DBA-4A9A-8863-0B23D8B7D37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4F2F41-4556-48C1-9346-689827FF17B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{1170B748-74A8-4F51-B865-6844E1F4A4D7}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
   <si>
     <t>6aabaf9b1896552dfac49667</t>
   </si>
@@ -195,6 +195,15 @@
   </si>
   <si>
     <t>Update Receive Status</t>
+  </si>
+  <si>
+    <t>Cancel Booking &amp; Rollback Inventory</t>
+  </si>
+  <si>
+    <t>excellent</t>
+  </si>
+  <si>
+    <t>You recognized the overload early, stepped back, came back with a clean policy decision (full cancellation only), safeguarded the financial ledger, wrote and tested every defensive condition in Postman, and caught every invalid boundary state before executing database persistence. Outstanding work.</t>
   </si>
 </sst>
 </file>
@@ -774,11 +783,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45C25416-15F1-45E5-92CA-5DD08DB17583}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="147.453125" bestFit="1" customWidth="1"/>
@@ -849,6 +858,23 @@
         <v>35</v>
       </c>
     </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>